<commit_message>
Changed the List of School
</commit_message>
<xml_diff>
--- a/public/data/schools.xlsx
+++ b/public/data/schools.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>schoolName</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>Check with us for More Listed Schools</t>
+  </si>
+  <si>
+    <t>Rutherford County Schools Only</t>
   </si>
   <si>
     <t>Blackman Middle School</t>
@@ -503,13 +506,17 @@
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>5</v>

</xml_diff>